<commit_message>
Fixed code for filtering movies and scraping IMDb attributes. Altered the code to automate the manual filtering decisions that I previously did.
</commit_message>
<xml_diff>
--- a/movie-release-optimization/data/processing/filter 1/xlsx/marvel_movies.xlsx
+++ b/movie-release-optimization/data/processing/filter 1/xlsx/marvel_movies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kitkat/github projects/Marvel-Analytics-by-KS/movie-release-optimization/data/cleaned/xlsx/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kitkat/github projects/Marvel-Analytics-by-KS/movie-release-optimization/data/processing/filter 1/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12786699-175B-0244-BE89-B24ACBB80725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9812037A-5997-2C44-B9C8-05B267B9CE8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="20" windowWidth="19220" windowHeight="21600" xr2:uid="{0EAFD10D-0BCC-FA4E-8446-8BA5CD0E0E58}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19220" windowHeight="18000" xr2:uid="{0EAFD10D-0BCC-FA4E-8446-8BA5CD0E0E58}"/>
   </bookViews>
   <sheets>
     <sheet name="marvel_movies" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="68">
   <si>
     <t>Iron Man</t>
   </si>
@@ -228,6 +228,15 @@
   </si>
   <si>
     <t>release_date</t>
+  </si>
+  <si>
+    <t>release_month</t>
+  </si>
+  <si>
+    <t>release_year</t>
+  </si>
+  <si>
+    <t>ISO_week</t>
   </si>
 </sst>
 </file>
@@ -763,7 +772,16 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="4">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     </dxf>
@@ -781,12 +799,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4F992C7A-5EAC-974A-A11F-B998F619FB8E}" name="Table1" displayName="Table1" ref="A1:C38" totalsRowShown="0">
-  <autoFilter ref="A1:C38" xr:uid="{4F992C7A-5EAC-974A-A11F-B998F619FB8E}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4F992C7A-5EAC-974A-A11F-B998F619FB8E}" name="Table1" displayName="Table1" ref="A1:F38" totalsRowShown="0">
+  <autoFilter ref="A1:F38" xr:uid="{4F992C7A-5EAC-974A-A11F-B998F619FB8E}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0DD13513-F771-024A-A1CD-D8CE8FBDEF89}" name="title"/>
-    <tableColumn id="2" xr3:uid="{CEC484DF-8126-B241-A1D6-6ADFACA33B11}" name="release_date" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{CEC484DF-8126-B241-A1D6-6ADFACA33B11}" name="release_date" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{F27F467F-F2C5-3D4A-8EDA-9BEA1680320D}" name="budget"/>
+    <tableColumn id="4" xr3:uid="{CF9D56C7-CE31-3C4C-AB98-D4979BA826C3}" name="release_month" dataDxfId="2">
+      <calculatedColumnFormula>MONTH(Table1[[#This Row],[release_date]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{DC2E2A6F-9A47-A74E-8AF6-FABEFDAE965E}" name="release_year" dataDxfId="1">
+      <calculatedColumnFormula>YEAR(Table1[[#This Row],[release_date]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{6AEC0E5F-5C2F-C344-8DB2-22CB71218D93}" name="ISO_week" dataDxfId="0">
+      <calculatedColumnFormula>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1109,15 +1136,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9175C09-312F-5C44-B538-879DE991E9FE}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="37.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="1.5" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>63</v>
       </c>
@@ -1127,8 +1154,17 @@
       <c r="C1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1138,8 +1174,20 @@
       <c r="C2" s="1">
         <v>140000000</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D2">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>5</v>
+      </c>
+      <c r="E2">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2008</v>
+      </c>
+      <c r="F2">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1149,8 +1197,20 @@
       <c r="C3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D3">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>6</v>
+      </c>
+      <c r="E3">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2008</v>
+      </c>
+      <c r="F3">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1160,8 +1220,20 @@
       <c r="C4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D4">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2010</v>
+      </c>
+      <c r="F4">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1171,8 +1243,20 @@
       <c r="C5" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D5">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2011</v>
+      </c>
+      <c r="F5">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1182,8 +1266,20 @@
       <c r="C6" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D6">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+      <c r="E6">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2011</v>
+      </c>
+      <c r="F6">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1193,8 +1289,20 @@
       <c r="C7" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D7">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2012</v>
+      </c>
+      <c r="F7">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1204,8 +1312,20 @@
       <c r="C8" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D8">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2013</v>
+      </c>
+      <c r="F8">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1215,8 +1335,20 @@
       <c r="C9" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D9">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>11</v>
+      </c>
+      <c r="E9">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2013</v>
+      </c>
+      <c r="F9">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1226,8 +1358,20 @@
       <c r="C10" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D10">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>4</v>
+      </c>
+      <c r="E10">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2014</v>
+      </c>
+      <c r="F10">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1237,8 +1381,20 @@
       <c r="C11" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D11">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>8</v>
+      </c>
+      <c r="E11">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2014</v>
+      </c>
+      <c r="F11">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1248,8 +1404,20 @@
       <c r="C12" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D12">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>5</v>
+      </c>
+      <c r="E12">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2015</v>
+      </c>
+      <c r="F12">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1259,8 +1427,20 @@
       <c r="C13" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D13">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+      <c r="E13">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2015</v>
+      </c>
+      <c r="F13">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1270,8 +1450,20 @@
       <c r="C14" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D14">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>5</v>
+      </c>
+      <c r="E14">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2016</v>
+      </c>
+      <c r="F14">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1281,8 +1473,20 @@
       <c r="C15" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D15">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>11</v>
+      </c>
+      <c r="E15">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2016</v>
+      </c>
+      <c r="F15">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1292,8 +1496,20 @@
       <c r="C16" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D16">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>5</v>
+      </c>
+      <c r="E16">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2017</v>
+      </c>
+      <c r="F16">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -1303,8 +1519,20 @@
       <c r="C17" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D17">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+      <c r="E17">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2017</v>
+      </c>
+      <c r="F17">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1314,8 +1542,20 @@
       <c r="C18" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D18">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>11</v>
+      </c>
+      <c r="E18">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2017</v>
+      </c>
+      <c r="F18">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1325,8 +1565,20 @@
       <c r="C19" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D19">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2018</v>
+      </c>
+      <c r="F19">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -1336,8 +1588,20 @@
       <c r="C20" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D20">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>4</v>
+      </c>
+      <c r="E20">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2018</v>
+      </c>
+      <c r="F20">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1347,8 +1611,20 @@
       <c r="C21" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D21">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+      <c r="E21">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2018</v>
+      </c>
+      <c r="F21">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -1358,8 +1634,20 @@
       <c r="C22" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D22">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>3</v>
+      </c>
+      <c r="E22">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2019</v>
+      </c>
+      <c r="F22">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1369,8 +1657,20 @@
       <c r="C23" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D23">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>4</v>
+      </c>
+      <c r="E23">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2019</v>
+      </c>
+      <c r="F23">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1380,8 +1680,20 @@
       <c r="C24" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D24">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+      <c r="E24">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2019</v>
+      </c>
+      <c r="F24">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1391,8 +1703,20 @@
       <c r="C25" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D25">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+      <c r="E25">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2021</v>
+      </c>
+      <c r="F25">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -1402,8 +1726,20 @@
       <c r="C26" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D26">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>9</v>
+      </c>
+      <c r="E26">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2021</v>
+      </c>
+      <c r="F26">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -1413,8 +1749,20 @@
       <c r="C27" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D27">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>11</v>
+      </c>
+      <c r="E27">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2021</v>
+      </c>
+      <c r="F27">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -1424,8 +1772,20 @@
       <c r="C28" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D28">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>12</v>
+      </c>
+      <c r="E28">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2021</v>
+      </c>
+      <c r="F28">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1435,8 +1795,20 @@
       <c r="C29" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D29">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>5</v>
+      </c>
+      <c r="E29">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2022</v>
+      </c>
+      <c r="F29">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -1446,8 +1818,20 @@
       <c r="C30" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D30">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+      <c r="E30">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2022</v>
+      </c>
+      <c r="F30">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -1457,8 +1841,20 @@
       <c r="C31" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D31">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>11</v>
+      </c>
+      <c r="E31">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2022</v>
+      </c>
+      <c r="F31">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -1468,8 +1864,20 @@
       <c r="C32" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D32">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>2</v>
+      </c>
+      <c r="E32">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2023</v>
+      </c>
+      <c r="F32">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -1479,8 +1887,20 @@
       <c r="C33" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D33">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>5</v>
+      </c>
+      <c r="E33">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2023</v>
+      </c>
+      <c r="F33">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -1490,8 +1910,20 @@
       <c r="C34" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D34">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>11</v>
+      </c>
+      <c r="E34">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2023</v>
+      </c>
+      <c r="F34">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -1501,8 +1933,20 @@
       <c r="C35" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D35">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+      <c r="E35">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2024</v>
+      </c>
+      <c r="F35">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -1512,8 +1956,20 @@
       <c r="C36" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D36">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>2</v>
+      </c>
+      <c r="E36">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2025</v>
+      </c>
+      <c r="F36">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>61</v>
       </c>
@@ -1523,8 +1979,20 @@
       <c r="C37" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D37">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>5</v>
+      </c>
+      <c r="E37">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2025</v>
+      </c>
+      <c r="F37">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>35</v>
       </c>
@@ -1533,6 +2001,18 @@
       </c>
       <c r="C38" t="s">
         <v>41</v>
+      </c>
+      <c r="D38">
+        <f>MONTH(Table1[[#This Row],[release_date]])</f>
+        <v>7</v>
+      </c>
+      <c r="E38">
+        <f>YEAR(Table1[[#This Row],[release_date]])</f>
+        <v>2025</v>
+      </c>
+      <c r="F38">
+        <f>_xlfn.ISOWEEKNUM(Table1[[#This Row],[release_date]])</f>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>